<commit_message>
feat: add CRC and USD patrimony amounts
</commit_message>
<xml_diff>
--- a/public/templates/patrimony-records-template.xlsx
+++ b/public/templates/patrimony-records-template.xlsx
@@ -50,7 +50,8 @@
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="36" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -66,10 +67,15 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t>Monto</t>
+          <t>Monto CRC</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t>Monto USD</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
         <is>
           <t>Nota</t>
         </is>

</xml_diff>

<commit_message>
feat: add patrimony record movement type
</commit_message>
<xml_diff>
--- a/public/templates/patrimony-records-template.xlsx
+++ b/public/templates/patrimony-records-template.xlsx
@@ -49,9 +49,10 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="36" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -67,15 +68,20 @@
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t>Monto CRC</t>
+          <t>Tipo de movimiento</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
+          <t>Monto CRC</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
           <t>Monto USD</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr" s="1">
+      <c r="F1" t="inlineStr" s="1">
         <is>
           <t>Nota</t>
         </is>

</xml_diff>